<commit_message>
Integrar evidencias al informe principal
</commit_message>
<xml_diff>
--- a/documentacion/entregables/Analisis_Riesgos.xlsx
+++ b/documentacion/entregables/Analisis_Riesgos.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz de Riesgos" sheetId="1" r:id="Rba1d757fb09e459f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" r:id="R937539d4daa9440a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="3" r:id="R0e70b16a97cd4492"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz de Riesgos" sheetId="1" r:id="R888f29bd57e64e67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" r:id="Re010dae1c6144a96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="3" r:id="Rb31f39e90a27487f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -542,73 +542,73 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="10" t="str">
-        <x:v>Aplicacion Flask</x:v>
+        <x:v>Servidor Fedora</x:v>
       </x:c>
       <x:c r="B10" s="10" t="str">
-        <x:v>Exposicion de informacion tecnica</x:v>
+        <x:v>Resolucion de nombres innecesaria</x:v>
       </x:c>
       <x:c r="C10" s="10" t="str">
-        <x:v>Modo debug activo</x:v>
+        <x:v>Puerto 5355/LLMNR abierto</x:v>
       </x:c>
       <x:c r="D10" s="12" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E10" s="12" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F10" s="12" t="n">
         <x:f>D10*E10</x:f>
-        <x:v>15</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G10" s="10" t="str">
-        <x:v>Alto</x:v>
+        <x:v>Medio</x:v>
       </x:c>
       <x:c r="H10" s="10" t="str">
-        <x:v>Desactivar debug fuera del laboratorio y usar servidor WSGI para produccion.</x:v>
+        <x:v>Deshabilitar LLMNR si no es requerido para el laboratorio.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="10" t="str">
-        <x:v>Sistema web</x:v>
+        <x:v>Aplicacion Flask</x:v>
       </x:c>
       <x:c r="B11" s="10" t="str">
-        <x:v>Acciones no autorizadas</x:v>
+        <x:v>Exposicion de informacion tecnica</x:v>
       </x:c>
       <x:c r="C11" s="10" t="str">
-        <x:v>Formularios sin token CSRF</x:v>
+        <x:v>Modo debug activo</x:v>
       </x:c>
       <x:c r="D11" s="12" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E11" s="12" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="F11" s="12" t="n">
         <x:f>D11*E11</x:f>
-        <x:v>9</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G11" s="10" t="str">
-        <x:v>Medio</x:v>
+        <x:v>Alto</x:v>
       </x:c>
       <x:c r="H11" s="10" t="str">
-        <x:v>Implementar CSRF tokens en formularios y validar origen de solicitudes.</x:v>
+        <x:v>Desactivar debug fuera del laboratorio y usar servidor WSGI para produccion.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="10" t="str">
-        <x:v>Servidor Fedora</x:v>
+        <x:v>Aplicacion Flask</x:v>
       </x:c>
       <x:c r="B12" s="10" t="str">
-        <x:v>Uso indebido de privilegios</x:v>
+        <x:v>Uso de servidor no productivo</x:v>
       </x:c>
       <x:c r="C12" s="10" t="str">
-        <x:v>Usuarios o servicios con permisos excesivos</x:v>
+        <x:v>Werkzeug Development Server expuesto</x:v>
       </x:c>
       <x:c r="D12" s="12" t="n">
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="E12" s="12" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F12" s="12" t="n">
         <x:f>D12*E12</x:f>
@@ -618,33 +618,141 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="H12" s="10" t="str">
-        <x:v>Principio de minimo privilegio y cuentas separadas para administracion.</x:v>
+        <x:v>Usar Gunicorn/uWSGI detras de Nginx o Apache en entornos reales.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="10" t="str">
-        <x:v>Sistema web y servidor</x:v>
+        <x:v>Servidor Fedora</x:v>
       </x:c>
       <x:c r="B13" s="10" t="str">
-        <x:v>Perdida de disponibilidad</x:v>
+        <x:v>Divulgacion de informacion temporal</x:v>
       </x:c>
       <x:c r="C13" s="10" t="str">
-        <x:v>Ausencia de procedimiento de respaldo</x:v>
+        <x:v>ICMP Timestamp Request habilitado</x:v>
       </x:c>
       <x:c r="D13" s="12" t="n">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E13" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="F13" s="12" t="n">
         <x:f>D13*E13</x:f>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="G13" s="10" t="str">
+        <x:v>Bajo</x:v>
+      </x:c>
+      <x:c r="H13" s="10" t="str">
+        <x:v>Filtrar o deshabilitar respuestas ICMP timestamp si no son necesarias.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="10" t="str">
+        <x:v>Sistema web</x:v>
+      </x:c>
+      <x:c r="B14" s="10" t="str">
+        <x:v>Debilidad en manejo de sesion</x:v>
+      </x:c>
+      <x:c r="C14" s="10" t="str">
+        <x:v>Cookies expiradas o sin endurecimiento suficiente</x:v>
+      </x:c>
+      <x:c r="D14" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E14" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F14" s="12" t="n">
+        <x:f>D14*E14</x:f>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G14" s="10" t="str">
+        <x:v>Medio</x:v>
+      </x:c>
+      <x:c r="H14" s="10" t="str">
+        <x:v>Configurar atributos Secure, HttpOnly, SameSite y expiracion adecuada.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="10" t="str">
+        <x:v>Sistema web</x:v>
+      </x:c>
+      <x:c r="B15" s="10" t="str">
+        <x:v>Acciones no autorizadas</x:v>
+      </x:c>
+      <x:c r="C15" s="10" t="str">
+        <x:v>Formularios sin token CSRF</x:v>
+      </x:c>
+      <x:c r="D15" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E15" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F15" s="12" t="n">
+        <x:f>D15*E15</x:f>
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G15" s="10" t="str">
+        <x:v>Medio</x:v>
+      </x:c>
+      <x:c r="H15" s="10" t="str">
+        <x:v>Implementar CSRF tokens en formularios y validar origen de solicitudes.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="10" t="str">
+        <x:v>Servidor Fedora</x:v>
+      </x:c>
+      <x:c r="B16" s="10" t="str">
+        <x:v>Uso indebido de privilegios</x:v>
+      </x:c>
+      <x:c r="C16" s="10" t="str">
+        <x:v>Usuarios o servicios con permisos excesivos</x:v>
+      </x:c>
+      <x:c r="D16" s="12" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E16" s="12" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="F16" s="12" t="n">
+        <x:f>D16*E16</x:f>
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="G16" s="10" t="str">
+        <x:v>Alto</x:v>
+      </x:c>
+      <x:c r="H16" s="10" t="str">
+        <x:v>Principio de minimo privilegio y cuentas separadas para administracion.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="10" t="str">
+        <x:v>Sistema web y servidor</x:v>
+      </x:c>
+      <x:c r="B17" s="10" t="str">
+        <x:v>Perdida de disponibilidad</x:v>
+      </x:c>
+      <x:c r="C17" s="10" t="str">
+        <x:v>Ausencia de procedimiento de respaldo</x:v>
+      </x:c>
+      <x:c r="D17" s="12" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E17" s="12" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="F17" s="12" t="n">
+        <x:f>D17*E17</x:f>
         <x:v>10</x:v>
       </x:c>
-      <x:c r="G13" s="10" t="str">
+      <x:c r="G17" s="10" t="str">
         <x:v>Medio</x:v>
       </x:c>
-      <x:c r="H13" s="10" t="str">
+      <x:c r="H17" s="10" t="str">
         <x:v>Copias periodicas de la base SQLite y del codigo fuente versionado.</x:v>
       </x:c>
     </x:row>
@@ -693,7 +801,7 @@
         <x:v>Critico</x:v>
       </x:c>
       <x:c r="B4" s="9" t="n">
-        <x:f>COUNTIF('Matriz de Riesgos'!G4:G13,A4)</x:f>
+        <x:f>COUNTIF('Matriz de Riesgos'!G4:G17,A4)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
@@ -708,8 +816,8 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="B5" s="9" t="n">
-        <x:f>COUNTIF('Matriz de Riesgos'!G4:G13,A5)</x:f>
-        <x:v>6</x:v>
+        <x:f>COUNTIF('Matriz de Riesgos'!G4:G17,A5)</x:f>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C5" s="9" t="str">
         <x:v>Riesgo importante</x:v>
@@ -723,8 +831,8 @@
         <x:v>Medio</x:v>
       </x:c>
       <x:c r="B6" s="9" t="n">
-        <x:f>COUNTIF('Matriz de Riesgos'!G4:G13,A6)</x:f>
-        <x:v>3</x:v>
+        <x:f>COUNTIF('Matriz de Riesgos'!G4:G17,A6)</x:f>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
         <x:v>Riesgo controlable</x:v>
@@ -738,8 +846,8 @@
         <x:v>Bajo</x:v>
       </x:c>
       <x:c r="B7" s="9" t="n">
-        <x:f>COUNTIF('Matriz de Riesgos'!G4:G13,A7)</x:f>
-        <x:v>0</x:v>
+        <x:f>COUNTIF('Matriz de Riesgos'!G4:G17,A7)</x:f>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C7" s="9" t="str">
         <x:v>Riesgo aceptable</x:v>

</xml_diff>

<commit_message>
Pulir informe y unificar analisis
</commit_message>
<xml_diff>
--- a/documentacion/entregables/Analisis_Riesgos.xlsx
+++ b/documentacion/entregables/Analisis_Riesgos.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz de Riesgos" sheetId="1" r:id="R888f29bd57e64e67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" r:id="Re010dae1c6144a96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="3" r:id="Rb31f39e90a27487f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz de Riesgos" sheetId="1" r:id="R5086b3f1aa2a446d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" r:id="Rcc4031f4e2d14689"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="3" r:id="R75e74317c48d4d79"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Crear documentos complementarios finales
</commit_message>
<xml_diff>
--- a/documentacion/entregables/Analisis_Riesgos.xlsx
+++ b/documentacion/entregables/Analisis_Riesgos.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz de Riesgos" sheetId="1" r:id="R5086b3f1aa2a446d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" r:id="Rcc4031f4e2d14689"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="3" r:id="R75e74317c48d4d79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz de Riesgos" sheetId="1" r:id="R2704fa47d1ed49ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" r:id="R846a4c20570d4b6b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Criterios" sheetId="3" r:id="R3bbb5c15f52849ea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="4" r:id="R510ba072379d4988"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -342,7 +343,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="13" t="str">
-        <x:v>Matriz de Analisis de Riesgos - Sistema de Ventas</x:v>
+        <x:v>Matriz de Análisis de Riesgos - Sistema de Ventas</x:v>
       </x:c>
       <x:c r="B1" s="14"/>
       <x:c r="C1" s="14"/>
@@ -386,7 +387,7 @@
         <x:v>Acceso no autorizado</x:v>
       </x:c>
       <x:c r="C4" s="10" t="str">
-        <x:v>Credenciales debiles y contrasenas predecibles</x:v>
+        <x:v>Credenciales débiles y contraseñas predecibles</x:v>
       </x:c>
       <x:c r="D4" s="12" t="n">
         <x:v>5</x:v>
@@ -399,10 +400,10 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="G4" s="10" t="str">
-        <x:v>Critico</x:v>
+        <x:v>Crítico</x:v>
       </x:c>
       <x:c r="H4" s="10" t="str">
-        <x:v>Politica de contrasenas, bloqueo por intentos fallidos y revision de usuarios.</x:v>
+        <x:v>Política de contraseñas, bloqueo por intentos fallidos y revisión de usuarios.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -410,10 +411,10 @@
         <x:v>Sistema web</x:v>
       </x:c>
       <x:c r="B5" s="10" t="str">
-        <x:v>Ingreso sin autenticacion valida</x:v>
+        <x:v>Ingreso sin autenticación válida</x:v>
       </x:c>
       <x:c r="C5" s="10" t="str">
-        <x:v>SQL injection en formulario de login</x:v>
+        <x:v>SQL Injection en formulario de login</x:v>
       </x:c>
       <x:c r="D5" s="12" t="n">
         <x:v>5</x:v>
@@ -429,7 +430,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="H5" s="10" t="str">
-        <x:v>Consultas parametrizadas, validacion de entradas y pruebas de seguridad.</x:v>
+        <x:v>Consultas parametrizadas, validación de entradas y pruebas de seguridad.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -437,10 +438,10 @@
         <x:v>Sistema web</x:v>
       </x:c>
       <x:c r="B6" s="10" t="str">
-        <x:v>Robo de sesion o ejecucion de scripts</x:v>
+        <x:v>Robo de sesión o ejecución de scripts</x:v>
       </x:c>
       <x:c r="C6" s="10" t="str">
-        <x:v>XSS reflejado en busqueda</x:v>
+        <x:v>XSS reflejado en búsqueda</x:v>
       </x:c>
       <x:c r="D6" s="12" t="n">
         <x:v>3</x:v>
@@ -464,10 +465,10 @@
         <x:v>Sistema web</x:v>
       </x:c>
       <x:c r="B7" s="10" t="str">
-        <x:v>Ejecucion persistente de JavaScript</x:v>
+        <x:v>Ejecución persistente de JavaScript</x:v>
       </x:c>
       <x:c r="C7" s="10" t="str">
-        <x:v>XSS almacenado en descripcion de productos</x:v>
+        <x:v>XSS almacenado en descripción de productos</x:v>
       </x:c>
       <x:c r="D7" s="12" t="n">
         <x:v>5</x:v>
@@ -483,7 +484,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="H7" s="10" t="str">
-        <x:v>No usar contenido de usuario como seguro, sanitizar y validar campos.</x:v>
+        <x:v>No usar contenido del usuario como HTML seguro; sanitizar y validar campos.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -491,10 +492,10 @@
         <x:v>Base de datos</x:v>
       </x:c>
       <x:c r="B8" s="10" t="str">
-        <x:v>Exposicion de credenciales</x:v>
+        <x:v>Exposición de credenciales</x:v>
       </x:c>
       <x:c r="C8" s="10" t="str">
-        <x:v>Contrasenas almacenadas en texto plano</x:v>
+        <x:v>Contraseñas almacenadas en texto plano</x:v>
       </x:c>
       <x:c r="D8" s="12" t="n">
         <x:v>5</x:v>
@@ -510,7 +511,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="H8" s="10" t="str">
-        <x:v>Hash seguro con bcrypt o argon2 y sal unica por usuario.</x:v>
+        <x:v>Hash seguro con bcrypt o argon2 y sal única por usuario.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -518,7 +519,7 @@
         <x:v>Servidor Fedora</x:v>
       </x:c>
       <x:c r="B9" s="10" t="str">
-        <x:v>Enumeracion de servicios</x:v>
+        <x:v>Enumeración de servicios</x:v>
       </x:c>
       <x:c r="C9" s="10" t="str">
         <x:v>Puerto 5000 expuesto durante el laboratorio</x:v>
@@ -537,7 +538,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="H9" s="10" t="str">
-        <x:v>Firewall, apertura temporal del puerto y cierre al finalizar la presentacion.</x:v>
+        <x:v>Firewall, apertura temporal del puerto y cierre al finalizar la presentación.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -545,7 +546,7 @@
         <x:v>Servidor Fedora</x:v>
       </x:c>
       <x:c r="B10" s="10" t="str">
-        <x:v>Resolucion de nombres innecesaria</x:v>
+        <x:v>Resolución de nombres innecesaria</x:v>
       </x:c>
       <x:c r="C10" s="10" t="str">
         <x:v>Puerto 5355/LLMNR abierto</x:v>
@@ -569,10 +570,10 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="10" t="str">
-        <x:v>Aplicacion Flask</x:v>
+        <x:v>Aplicación Flask</x:v>
       </x:c>
       <x:c r="B11" s="10" t="str">
-        <x:v>Exposicion de informacion tecnica</x:v>
+        <x:v>Exposición de información técnica</x:v>
       </x:c>
       <x:c r="C11" s="10" t="str">
         <x:v>Modo debug activo</x:v>
@@ -591,12 +592,12 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="H11" s="10" t="str">
-        <x:v>Desactivar debug fuera del laboratorio y usar servidor WSGI para produccion.</x:v>
+        <x:v>Desactivar debug fuera del laboratorio y usar servidor WSGI para producción.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="10" t="str">
-        <x:v>Aplicacion Flask</x:v>
+        <x:v>Aplicación Flask</x:v>
       </x:c>
       <x:c r="B12" s="10" t="str">
         <x:v>Uso de servidor no productivo</x:v>
@@ -618,7 +619,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="H12" s="10" t="str">
-        <x:v>Usar Gunicorn/uWSGI detras de Nginx o Apache en entornos reales.</x:v>
+        <x:v>Usar Gunicorn/uWSGI detrás de Nginx o Apache en entornos reales.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -626,7 +627,7 @@
         <x:v>Servidor Fedora</x:v>
       </x:c>
       <x:c r="B13" s="10" t="str">
-        <x:v>Divulgacion de informacion temporal</x:v>
+        <x:v>Divulgación de información temporal</x:v>
       </x:c>
       <x:c r="C13" s="10" t="str">
         <x:v>ICMP Timestamp Request habilitado</x:v>
@@ -653,7 +654,7 @@
         <x:v>Sistema web</x:v>
       </x:c>
       <x:c r="B14" s="10" t="str">
-        <x:v>Debilidad en manejo de sesion</x:v>
+        <x:v>Debilidad en manejo de sesión</x:v>
       </x:c>
       <x:c r="C14" s="10" t="str">
         <x:v>Cookies expiradas o sin endurecimiento suficiente</x:v>
@@ -672,7 +673,7 @@
         <x:v>Medio</x:v>
       </x:c>
       <x:c r="H14" s="10" t="str">
-        <x:v>Configurar atributos Secure, HttpOnly, SameSite y expiracion adecuada.</x:v>
+        <x:v>Configurar atributos Secure, HttpOnly, SameSite y expiración adecuada.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -726,7 +727,7 @@
         <x:v>Alto</x:v>
       </x:c>
       <x:c r="H16" s="10" t="str">
-        <x:v>Principio de minimo privilegio y cuentas separadas para administracion.</x:v>
+        <x:v>Principio de mínimo privilegio y cuentas separadas para administración.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -734,7 +735,7 @@
         <x:v>Sistema web y servidor</x:v>
       </x:c>
       <x:c r="B17" s="10" t="str">
-        <x:v>Perdida de disponibilidad</x:v>
+        <x:v>Pérdida de disponibilidad</x:v>
       </x:c>
       <x:c r="C17" s="10" t="str">
         <x:v>Ausencia de procedimiento de respaldo</x:v>
@@ -753,7 +754,7 @@
         <x:v>Medio</x:v>
       </x:c>
       <x:c r="H17" s="10" t="str">
-        <x:v>Copias periodicas de la base SQLite y del codigo fuente versionado.</x:v>
+        <x:v>Copias periódicas de la base SQLite y del código fuente versionado.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -790,22 +791,22 @@
         <x:v>Cantidad</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
-        <x:v>Interpretacion</x:v>
+        <x:v>Interpretación</x:v>
       </x:c>
       <x:c r="D3" s="6" t="str">
-        <x:v>Accion sugerida</x:v>
+        <x:v>Acción sugerida</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="9" t="str">
-        <x:v>Critico</x:v>
+        <x:v>Crítico</x:v>
       </x:c>
       <x:c r="B4" s="9" t="n">
         <x:f>COUNTIF('Matriz de Riesgos'!G4:G17,A4)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C4" s="9" t="str">
-        <x:v>Requiere atencion inmediata</x:v>
+        <x:v>Requiere atención inmediata</x:v>
       </x:c>
       <x:c r="D4" s="9" t="str">
         <x:v>Corregir antes de exponer el sistema.</x:v>
@@ -823,7 +824,7 @@
         <x:v>Riesgo importante</x:v>
       </x:c>
       <x:c r="D5" s="9" t="str">
-        <x:v>Planificar mitigacion prioritaria.</x:v>
+        <x:v>Planificar mitigación prioritaria.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -868,6 +869,96 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="48" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="13" t="str">
+        <x:v>Criterios usados para impacto y probabilidad</x:v>
+      </x:c>
+      <x:c r="B1" s="14"/>
+      <x:c r="C1" s="14"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="6" t="str">
+        <x:v>Valor</x:v>
+      </x:c>
+      <x:c r="B3" s="6" t="str">
+        <x:v>Impacto</x:v>
+      </x:c>
+      <x:c r="C3" s="6" t="str">
+        <x:v>Probabilidad</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B4" s="10" t="str">
+        <x:v>Impacto muy bajo: efecto menor o fácilmente recuperable.</x:v>
+      </x:c>
+      <x:c r="C4" s="10" t="str">
+        <x:v>Muy improbable: requiere condiciones poco realistas.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="10" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B5" s="10" t="str">
+        <x:v>Impacto bajo: afecta parcialmente una función.</x:v>
+      </x:c>
+      <x:c r="C5" s="10" t="str">
+        <x:v>Poco probable: podría ocurrir, pero no es habitual.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="10" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B6" s="10" t="str">
+        <x:v>Impacto medio: afecta datos o disponibilidad de forma limitada.</x:v>
+      </x:c>
+      <x:c r="C6" s="10" t="str">
+        <x:v>Probable: puede ocurrir durante el uso normal o con pruebas básicas.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="10" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B7" s="10" t="str">
+        <x:v>Impacto alto: compromete funciones importantes del sistema.</x:v>
+      </x:c>
+      <x:c r="C7" s="10" t="str">
+        <x:v>Muy probable: puede repetirse con facilidad.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="10" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B8" s="10" t="str">
+        <x:v>Impacto crítico: compromete acceso, datos sensibles o continuidad.</x:v>
+      </x:c>
+      <x:c r="C8" s="10" t="str">
+        <x:v>Casi seguro: se explota con pasos simples o credenciales conocidas.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:C1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="78" hidden="0" customWidth="1"/>
   </x:cols>

</xml_diff>